<commit_message>
Texty lekcií: návrhy pre obrazovky 1 až 17 a 36
129 prepísaných textov — úvodné vety, zadania, vysvetlenia pri
odpovediach, poučky aj popisky dôkazových obrázkov. Krátke popisky,
ktoré musia zostať krátke (názvy políčok, možnosti v triedení), sa
zámerne nerozpisujú — rozbilo by to rozloženie obrazovky.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dokumenty/texty-lekcii.xlsx
+++ b/dokumenty/texty-lekcii.xlsx
@@ -788,9 +788,9 @@
           <t>Umelá inteligencia ako pomocník pri dôležitých finančných rozhodnutiach.</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia ako pomocník, ktorý vám pomôže rozpoznať podvod a rozumieť tomu, čo vám niekto posiela alebo ponúka.</t>
         </is>
       </c>
       <c r="F3" s="10" t="inlineStr"/>
@@ -817,9 +817,9 @@
           <t>Čaká vás 36 krátkych zastavení rozdelených do 5 častí. Pri každom si niečo vyskúšate a hneď sa dozviete, či ste odpovedali správne — aj prečo. Nič sa nedá pokaziť a kedykoľvek sa môžete vrátiť tam, kde ste skončili.</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>Čaká vás 36 krátkych zastavení rozdelených do 5 častí. Pri každom si niečo vyskúšate a hneď sa dozviete, či ste odpovedali správne — a hlavne prečo. Nemusíte sa báť, že niečo pokazíte: nič sa nedá rozbiť a za nesprávnu odpoveď vás nikto nehodnotí. Kurz môžete kedykoľvek zavrieť a nabudúce pokračovať presne tam, kde ste skončili.</t>
         </is>
       </c>
       <c r="F4" s="10" t="inlineStr"/>
@@ -846,9 +846,9 @@
           <t>Prezrite si päť častí kurzu nižšie a potom kliknite na tlačidlo &lt;strong&gt;„Ďalej“&lt;/strong&gt; v pravom dolnom rohu.</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>Prezrite si päť častí kurzu nižšie — uvidíte, čo vás čaká. Potom pokračujte kliknutím na tlačidlo &lt;strong&gt;„Ďalej“&lt;/strong&gt; v pravom dolnom rohu.</t>
         </is>
       </c>
       <c r="F5" s="10" t="inlineStr"/>
@@ -904,9 +904,9 @@
           <t>Päť tém, ktoré spolu prejdeme — od zoznámenia s AI až po zlaté pravidlá bezpečnosti.</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E7" s="11" t="inlineStr">
+        <is>
+          <t>Prejdeme spolu päť tém. Začneme zoznámením s umelou inteligenciou a skončíme pri zlatých pravidlách, ktoré vás ochránia aj bez nej.</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr"/>
@@ -933,9 +933,9 @@
           <t>Kliknite postupne na &lt;strong&gt;aspoň tri dlaždice&lt;/strong&gt;. Každá sa otvorí a ukáže, čo vás v danej časti čaká.</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E8" s="11" t="inlineStr">
+        <is>
+          <t>Kliknite postupne na &lt;strong&gt;aspoň tri dlaždice&lt;/strong&gt;. Každá sa otvorí a v krátkosti ukáže, čo sa v danej časti naučíte. Pokojne si otvorte všetkých päť.</t>
         </is>
       </c>
       <c r="F8" s="10" t="inlineStr"/>
@@ -1107,9 +1107,9 @@
           <t>Čo je umelá inteligencia, čo vie a čo nevie — a ako s ňou začať.</t>
         </is>
       </c>
-      <c r="E14" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E14" s="11" t="inlineStr">
+        <is>
+          <t>Vysvetlíme si jednoducho, čo umelá inteligencia je, v čom vám vie pomôcť a kde má hranice. Ukážeme si aj to, ako ju bezpečne získať a položiť jej prvú otázku.</t>
         </is>
       </c>
       <c r="F14" s="10" t="inlineStr"/>
@@ -1136,9 +1136,9 @@
           <t>Prečo si dôležité veci treba overiť aj z druhého zdroja.</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia si občas vymyslí odpoveď a tvári sa pritom úplne isto. Naučíte sa spoznať, kedy jej môžete veriť a kedy si treba informáciu overiť ešte niekde inde.</t>
         </is>
       </c>
       <c r="F15" s="10" t="inlineStr"/>
@@ -1165,9 +1165,9 @@
           <t>Podozrivé e-maily, telefonáty aj SMS — skutočné príklady zo života.</t>
         </is>
       </c>
-      <c r="E16" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Prezrieme si skutočné podvodné e-maily, SMS správy aj telefonáty, aké chodia ľuďom každý deň. Naučíte sa v nich nájsť varovné znaky skôr, než na niečo kliknete.</t>
         </is>
       </c>
       <c r="F16" s="10" t="inlineStr"/>
@@ -1194,9 +1194,9 @@
           <t>Poplašné správy, fotografie vytvorené AI a zložité zmluvy.</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E17" s="11" t="inlineStr">
+        <is>
+          <t>Ukážeme si poplašné správy zo sociálnych sietí, fotografie vyrobené umelou inteligenciou a to, ako si dať zložitú zmluvu vysvetliť v zrozumiteľnej reči.</t>
         </is>
       </c>
       <c r="F17" s="10" t="inlineStr"/>
@@ -1223,9 +1223,9 @@
           <t>Čo nikdy nikomu nezadávame — ani umelej inteligencii.</t>
         </is>
       </c>
-      <c r="E18" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E18" s="11" t="inlineStr">
+        <is>
+          <t>Zhrnieme si, ktoré údaje nepatria nikam — ani do umelej inteligencie. A povieme si, čo robiť, ak sa aj napriek opatrnosti niečo stane.</t>
         </is>
       </c>
       <c r="F18" s="10" t="inlineStr"/>
@@ -1281,9 +1281,9 @@
           <t>Predstavte si ju ako veľmi sčítaného pomocníka, ktorý ochotne poradí — ale volant držíte vy.</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>Predstavte si veľmi sčítaného pomocníka, ktorý ochotne poradí, vysvetlí a nikdy sa neurazí. Rozhodnutie však vždy zostáva na vás — volant držíte vy.</t>
         </is>
       </c>
       <c r="F20" s="10" t="inlineStr"/>
@@ -1310,9 +1310,9 @@
           <t>Kliknite postupne na &lt;strong&gt;všetky štyri karty&lt;/strong&gt;. Každá sa otočí a ukáže vysvetlenie na druhej strane.</t>
         </is>
       </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>Kliknite postupne na &lt;strong&gt;všetky štyri karty&lt;/strong&gt;. Každá sa otočí a na druhej strane nájdete krátke vysvetlenie. Ak si ju chcete prečítať znova, kliknite na ňu ešte raz.</t>
         </is>
       </c>
       <c r="F21" s="10" t="inlineStr"/>
@@ -1455,9 +1455,9 @@
           <t>AI si prečítala obrovské množstvo kníh, novín a webových stránok. Vďaka tomu vie odpovedať na otázky, vysvetľovať a radiť.</t>
         </is>
       </c>
-      <c r="E26" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia si prečítala obrovské množstvo kníh, novín a internetových stránok. Vďaka tomu vie odpovedať na otázky, vysvetľovať odborné pojmy a radiť — podobne, ako keby ste sa pýtali veľmi načítaného známeho.</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr"/>
@@ -1484,9 +1484,9 @@
           <t>Môžete sa jej pýtať kedykoľvek, koľkokrát chcete, a nikdy ju to neomrzí ani neurazí. Nemusíte sa báť, že otravujete.</t>
         </is>
       </c>
-      <c r="E27" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>Môžete sa jej pýtať kedykoľvek — ráno, večer, cez sviatky — a koľkokrát chcete. Nikdy ju to neomrzí a nikdy sa neurazí. Nemusíte mať pocit, že niekoho otravujete alebo že je vaša otázka hlúpa.</t>
         </is>
       </c>
       <c r="F27" s="10" t="inlineStr"/>
@@ -1513,9 +1513,9 @@
           <t>Podobne ako človek. Nie všetko, čo AI povie, je nutne pravda — dôležité veci si preto vždy overte.</t>
         </is>
       </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E28" s="7" t="inlineStr">
+        <is>
+          <t>Mýli sa podobne ako človek — s tým rozdielom, že to na nej nie je vidieť. Nie všetko, čo umelá inteligencia povie, musí byť pravda, preto si dôležité veci vždy overte aj inde.</t>
         </is>
       </c>
       <c r="F28" s="10" t="inlineStr"/>
@@ -1542,9 +1542,9 @@
           <t>Prvý program, ktorý viedol rozhovor podobný ľudskému, sa volal ELIZA a vznikol už v roku 1966. Umelá inteligencia teda nie je až taká nová vec.</t>
         </is>
       </c>
-      <c r="E29" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>Prvý program, ktorý dokázal viesť rozhovor podobný ľudskému, sa volal ELIZA a vznikol už v roku 1966 — teda pred šesťdesiatimi rokmi. Umelá inteligencia teda nie je žiadna novinka posledných rokov, len sa jej dnes darí oveľa lepšie.</t>
         </is>
       </c>
       <c r="F29" s="10" t="inlineStr"/>
@@ -1600,9 +1600,9 @@
           <t>Aby vám umelá inteligencia naozaj pomohla, treba vedieť, čo od nej môžete čakať — a čo už nie.</t>
         </is>
       </c>
-      <c r="E31" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Aby vám umelá inteligencia naozaj pomohla, treba vedieť, čo od nej môžete čakať a čo už nie. Práve v tom je rozdiel medzi užitočným pomocníkom a sklamaním.</t>
         </is>
       </c>
       <c r="F31" s="10" t="inlineStr"/>
@@ -1629,9 +1629,9 @@
           <t>Máte 10 kartičiek. Kliknite na kartičku a potom na políčko &lt;strong&gt;„AI vie“&lt;/strong&gt; alebo &lt;strong&gt;„AI nevie“&lt;/strong&gt;, kam podľa vás patrí. Pri každej vám hneď vysvetlíme, či ste sa trafili.</t>
         </is>
       </c>
-      <c r="E32" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Máte 10 kartičiek. Kliknite na kartičku a potom na políčko &lt;strong&gt;„AI vie“&lt;/strong&gt; alebo &lt;strong&gt;„AI nevie“&lt;/strong&gt; podľa toho, kam si myslíte, že patrí. Pri každej vám hneď vysvetlíme, či ste sa trafili — a nič sa nestane, ak sa pomýlite.</t>
         </is>
       </c>
       <c r="F32" s="10" t="inlineStr"/>
@@ -1948,9 +1948,9 @@
           <t>Toto je jedna z najsilnejších stránok AI — dokáže preložiť odbornú reč do zrozumiteľnej slovenčiny.</t>
         </is>
       </c>
-      <c r="E43" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>Toto je jedna z najsilnejších stránok umelej inteligencie. Dokáže vziať odborný text — zmluvu, list z úradu, poistné podmienky — a prerozprávať ho bežnou rečou. Pokojne ju požiadajte: „Vysvetli mi to ako pre začiatočníka.“</t>
         </is>
       </c>
       <c r="F43" s="10" t="inlineStr"/>
@@ -1977,9 +1977,9 @@
           <t>AI pozná typické znaky podvodov a vie vás na ne upozorniť skôr, než niečo podpíšete.</t>
         </is>
       </c>
-      <c r="E44" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia pozná typické znaky podvodov, lebo ich videla tisíce. Vie vás na ne upozorniť skôr, než niekam kliknete alebo niečo podpíšete — a upozorní aj na to, čo by vám samému nemuselo udrieť do očí.</t>
         </is>
       </c>
       <c r="F44" s="10" t="inlineStr"/>
@@ -2006,9 +2006,9 @@
           <t>Stačí jej správu prepísať alebo odfotiť a opýtať sa: „Je to podvod?“</t>
         </is>
       </c>
-      <c r="E45" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E45" s="11" t="inlineStr">
+        <is>
+          <t>Stačí jej podozrivú správu prepísať alebo odfotiť a opýtať sa: „Je toto podvod? Podľa čoho to spoznám?“ Odpoveď dostanete o pár sekúnd a rovno aj vysvetlenie, čoho si všímať nabudúce.</t>
         </is>
       </c>
       <c r="F45" s="10" t="inlineStr"/>
@@ -2035,9 +2035,9 @@
           <t>Z dvadsiatich strán vám AI spraví pár bodov s tým najdôležitejším.</t>
         </is>
       </c>
-      <c r="E46" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>Z dvadsiatich strán vám umelá inteligencia spraví pár bodov s tým najdôležitejším. Hodí sa to pri zmluvách, poistkách či podmienkach, ktoré by inak nikto nedočítal do konca.</t>
         </is>
       </c>
       <c r="F46" s="10" t="inlineStr"/>
@@ -2064,9 +2064,9 @@
           <t>Môžete sa pýtať koľkokrát chcete — AI sa nikdy neurazí ani neunaví.</t>
         </is>
       </c>
-      <c r="E47" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>Môžete sa pýtať koľkokrát chcete a tú istú otázku pokojne aj päťkrát za sebou. Umelá inteligencia sa neunaví ani neurazí. Ak odpovedi nerozumiete, jednoducho napíšte: „Vysvetli mi to jednoduchšie.“</t>
         </is>
       </c>
       <c r="F47" s="10" t="inlineStr"/>
@@ -2093,9 +2093,9 @@
           <t>AI môže poradiť, ale rozhodnutie — najmä pri peniazoch — musíte urobiť vy sami.</t>
         </is>
       </c>
-      <c r="E48" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia môže poradiť, ale rozhodnutie zostáva na vás — a pri peniazoch to platí dvojnásobne. Berte jej odpoveď ako názor známeho, nie ako pokyn, ktorý treba splniť.</t>
         </is>
       </c>
       <c r="F48" s="10" t="inlineStr"/>
@@ -2122,9 +2122,9 @@
           <t>AI sa občas mýli a tvári sa pritom veľmi presvedčivo. Preto sa dôležité fakty overujú.</t>
         </is>
       </c>
-      <c r="E49" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia sa občas mýli a tvári sa pritom rovnako isto ako vtedy, keď má pravdu. Práve preto sa dôležité údaje — čísla, dátumy, telefónne linky — vždy overujú ešte niekde inde.</t>
         </is>
       </c>
       <c r="F49" s="10" t="inlineStr"/>
@@ -2151,9 +2151,9 @@
           <t>AI je pomocník, nie odborník s licenciou. Pri vážnych veciach vždy oslovte skutočného profesionála.</t>
         </is>
       </c>
-      <c r="E50" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia je pomocník, nie odborník s licenciou a zodpovednosťou. Pri zdraví, súde alebo väčších peniazoch vám pomôže pripraviť sa a rozumieť pojmom, ale posledné slovo má lekár, právnik či váš bankár.</t>
         </is>
       </c>
       <c r="F50" s="10" t="inlineStr"/>
@@ -2180,9 +2180,9 @@
           <t>AI nemá prístup k vašim účtom ani peniazom — a to je dobre, chráni vás to.</t>
         </is>
       </c>
-      <c r="E51" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia sa nevie pozrieť do vášho účtu ani s ním nič urobiť — a to je dobre, práve to vás chráni. Ak by od vás niekto pýtal prístup do banky „pre umelú inteligenciu“, je to podvod.</t>
         </is>
       </c>
       <c r="F51" s="10" t="inlineStr"/>
@@ -2209,9 +2209,9 @@
           <t>Ak sa niečo pokazí, AI za to neručí. Zodpovednosť zostáva vždy na človeku.</t>
         </is>
       </c>
-      <c r="E52" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E52" s="11" t="inlineStr">
+        <is>
+          <t>Ak sa niečo pokazí, umelá inteligencia za to neručí a nikto vám peniaze nevráti preto, že „to tak povedala AI“. Zodpovednosť zostáva vždy na človeku, ktorý stlačil tlačidlo.</t>
         </is>
       </c>
       <c r="F52" s="10" t="inlineStr"/>
@@ -2296,9 +2296,9 @@
           <t>Vysvetliť, zhrnúť, upozorniť, poradiť.</t>
         </is>
       </c>
-      <c r="E55" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E55" s="11" t="inlineStr">
+        <is>
+          <t>Vysvetliť, zhrnúť, upozorniť a poradiť.</t>
         </is>
       </c>
       <c r="F55" s="10" t="inlineStr"/>
@@ -2325,9 +2325,9 @@
           <t>Rozhodnúť za vás ani ručiť za správnosť.</t>
         </is>
       </c>
-      <c r="E56" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E56" s="11" t="inlineStr">
+        <is>
+          <t>Rozhodnúť za vás ani ručiť za to, že má pravdu.</t>
         </is>
       </c>
       <c r="F56" s="10" t="inlineStr"/>
@@ -2383,9 +2383,9 @@
           <t>AI je výborná na vysvetľovanie a upozorňovanie na riziká.</t>
         </is>
       </c>
-      <c r="E58" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E58" s="11" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia je výborná na vysvetľovanie a na upozorňovanie na riziká.</t>
         </is>
       </c>
       <c r="F58" s="10" t="inlineStr"/>
@@ -2412,9 +2412,9 @@
           <t>AI nikdy nepreberá zodpovednosť za vaše rozhodnutie.</t>
         </is>
       </c>
-      <c r="E59" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E59" s="11" t="inlineStr">
+        <is>
+          <t>Zodpovednosť za rozhodnutie nepreberá — tá zostáva vždy na vás.</t>
         </is>
       </c>
       <c r="F59" s="10" t="inlineStr"/>
@@ -2441,9 +2441,9 @@
           <t>Pri peniazoch je AI len prvý názor — nie posledné slovo.</t>
         </is>
       </c>
-      <c r="E60" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E60" s="11" t="inlineStr">
+        <is>
+          <t>Pri peniazoch berte jej odpoveď ako prvý názor, nie ako posledné slovo.</t>
         </is>
       </c>
       <c r="F60" s="10" t="inlineStr"/>
@@ -2470,9 +2470,9 @@
           <t>AI je ako navigácia v aute: dokáže vás skvele navigovať, ale volant držíte vy.</t>
         </is>
       </c>
-      <c r="E61" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E61" s="11" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia je ako navigácia v aute: poradí vám cestu, upozorní na zápchu, ale volant držíte vy. A keď vám povie, aby ste odbočili do rieky, jednoducho ju neposlúchnete.</t>
         </is>
       </c>
       <c r="F61" s="10" t="inlineStr"/>
@@ -2528,9 +2528,9 @@
           <t>Pri dôležitých veciach sa hovorí: vypočujte si aj názor niekoho druhého. AI je taký druhý názor na počkanie — zadarmo a bez toho, aby ste niekoho obťažovali.</t>
         </is>
       </c>
-      <c r="E63" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>Pri dôležitých veciach sa hovorí: vypočujte si aj názor niekoho druhého. Umelá inteligencia je presne taký druhý názor na počkanie — kedykoľvek, zadarmo a bez pocitu, že niekoho zdržiavate.</t>
         </is>
       </c>
       <c r="F63" s="10" t="inlineStr"/>
@@ -2557,9 +2557,9 @@
           <t>Kliknite na situáciu &lt;strong&gt;vľavo&lt;/strong&gt; a potom na políčko &lt;strong&gt;vpravo&lt;/strong&gt;, ktoré k nej patrí. Ak sa trafíte, spojí ich čiara.</t>
         </is>
       </c>
-      <c r="E64" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Kliknite najprv na situáciu &lt;strong&gt;vľavo&lt;/strong&gt; a potom na políčko &lt;strong&gt;vpravo&lt;/strong&gt;, ktoré k nej podľa vás patrí. Ak sa trafíte, spojí ich čiara. Ak nie, skúste to jednoducho znova.</t>
         </is>
       </c>
       <c r="F64" s="10" t="inlineStr"/>
@@ -2702,9 +2702,9 @@
           <t>Rozoberie ho vetu po vete a ukáže varovné znaky.</t>
         </is>
       </c>
-      <c r="E69" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Rozoberie ho vetu po vete a ukáže varovné znaky.</t>
         </is>
       </c>
       <c r="F69" s="10" t="inlineStr"/>
@@ -2818,9 +2818,9 @@
           <t>AI si prejde text a upozorní na časový nátlak, podozrivé odkazy či zvláštnu adresu odosielateľa.</t>
         </is>
       </c>
-      <c r="E73" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia si text prejde vetu po vete a upozorní na časový nátlak, podozrivé odkazy aj na zvláštnu adresu odosielateľa. Ukáže vám teda nielen to, že ide o podvod, ale aj podľa čoho ste to mohli spoznať sami.</t>
         </is>
       </c>
       <c r="F73" s="10" t="inlineStr"/>
@@ -2847,9 +2847,9 @@
           <t>Dozviete sa, že banka nikdy nežiada PIN ani prevod na „bezpečný účet“ — a hneď viete, že šlo o podvod.</t>
         </is>
       </c>
-      <c r="E74" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>Dozviete sa, ako banka v takej situácii naozaj postupuje: nikdy nepýta PIN a nikdy nežiada previesť peniaze na takzvaný „bezpečný účet“. Keď to viete, spoznáte podvod už počas hovoru.</t>
         </is>
       </c>
       <c r="F74" s="10" t="inlineStr"/>
@@ -2876,9 +2876,9 @@
           <t>AI vám pripraví zoznam otázok pre predajcu — napríklad na poplatky, licenciu a možnosť výberu peňazí.</t>
         </is>
       </c>
-      <c r="E75" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia vám pripraví zoznam otázok, ktoré sa oplatí položiť — na poplatky, na licenciu od Národnej banky a na to, ako sa dajú peniaze vybrať späť. Podvodník sa pri takých otázkach zvyčajne začne vyhýbať odpovedi.</t>
         </is>
       </c>
       <c r="F75" s="10" t="inlineStr"/>
@@ -2905,9 +2905,9 @@
           <t>Z právnickej reči spraví ľudskú — a upozorní na pokuty či automatické predĺženie.</t>
         </is>
       </c>
-      <c r="E76" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>Z právnickej reči spraví ľudskú a upozorní na miesta, ktoré sa ľahko prehliadnu — pokuty, výpovedné lehoty či automatické predĺženie zmluvy o ďalší rok.</t>
         </is>
       </c>
       <c r="F76" s="10" t="inlineStr"/>
@@ -2934,9 +2934,9 @@
           <t>Umelá inteligencia nie je neomylná. Pomôže vám premýšľať, no nenahrádza odborníka.</t>
         </is>
       </c>
-      <c r="E77" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia nie je neomylná a nie je odborník. Pomôže vám zorientovať sa a premýšľať nad správnymi otázkami — ale pri vážnych veciach sa vždy poraďte aj so skutočným človekom.</t>
         </is>
       </c>
       <c r="F77" s="10" t="inlineStr"/>
@@ -2992,9 +2992,9 @@
           <t>ChatGPT je najznámejšia aplikácia na prácu s umelou inteligenciou. Takto vyzerá na tablete — zoznámime sa s tromi miestami, ktoré budete používať najčastejšie.</t>
         </is>
       </c>
-      <c r="E79" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E79" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT je najznámejšia aplikácia na prácu s umelou inteligenciou. Takto vyzerá na tablete a rovnako vyzerá aj na telefóne či v počítači. Zoznámime sa s tromi miestami, ktoré budete používať najčastejšie — viac ich na začiatok naozaj netreba.</t>
         </is>
       </c>
       <c r="F79" s="10" t="inlineStr"/>
@@ -3021,9 +3021,9 @@
           <t>Na obrázku sú &lt;strong&gt;tri očíslované body&lt;/strong&gt;. Kliknite postupne na každý z nich — pod obrázkom sa im rozsvieti vysvetlenie.</t>
         </is>
       </c>
-      <c r="E80" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E80" s="11" t="inlineStr">
+        <is>
+          <t>Na obrázku sú &lt;strong&gt;tri očíslované body&lt;/strong&gt;. Kliknite postupne na každý z nich — pod obrázkom sa vám ku každému ukáže vysvetlenie, čo na tom mieste nájdete.</t>
         </is>
       </c>
       <c r="F80" s="10" t="inlineStr"/>
@@ -3137,9 +3137,9 @@
           <t>Vľavo — staršie otázky sa nestrácajú, kedykoľvek sa k nim vrátite.</t>
         </is>
       </c>
-      <c r="E84" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E84" s="11" t="inlineStr">
+        <is>
+          <t>Vľavo je zoznam vašich starších rozhovorov. Nič sa nestráca — kedykoľvek si môžete otvoriť, na čo ste sa pýtali minulý týždeň, a pokračovať tam, kde ste prestali.</t>
         </is>
       </c>
       <c r="F84" s="10" t="inlineStr"/>
@@ -3166,9 +3166,9 @@
           <t>Dole — otázka sa píše rovnako ako SMS správa.</t>
         </is>
       </c>
-      <c r="E85" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E85" s="11" t="inlineStr">
+        <is>
+          <t>Dole je okienko, do ktorého píšete otázku. Funguje presne ako písanie SMS správy — napíšete text a odošlete ho šípkou vedľa.</t>
         </is>
       </c>
       <c r="F85" s="10" t="inlineStr"/>
@@ -3195,9 +3195,9 @@
           <t>AI odpovie prehľadne, väčšinou v bodoch — tu napríklad rozpísaný plán výletu.</t>
         </is>
       </c>
-      <c r="E86" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E86" s="11" t="inlineStr">
+        <is>
+          <t>V hlavnej časti sa objaví odpoveď, zvyčajne prehľadne rozpísaná do bodov — tu napríklad plán výletu. Ak je odpoveď dlhá, pokojne požiadajte: „Zhrň mi to do troch viet.“</t>
         </is>
       </c>
       <c r="F86" s="10" t="inlineStr"/>
@@ -3224,9 +3224,9 @@
           <t>Skutočná obrazovka aplikácie ChatGPT na tablete — presne takto to uvidíte aj vy.</t>
         </is>
       </c>
-      <c r="E87" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E87" s="11" t="inlineStr">
+        <is>
+          <t>Toto nie je nákres, ale skutočná obrazovka aplikácie ChatGPT na tablete. Presne takto to uvidíte aj vy, keď si ju otvoríte.</t>
         </is>
       </c>
       <c r="F87" s="10" t="inlineStr"/>
@@ -3311,9 +3311,9 @@
           <t>Falošných napodobenín ChatGPT je v obchodoch s aplikáciami mnoho. Líšia sa drobnosťou v názve, majú podobné logo a pýtajú predplatné. Ukážeme si, ako spoznáte tú pravú.</t>
         </is>
       </c>
-      <c r="E90" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>V obchodoch s aplikáciami je množstvo napodobenín ChatGPT. Líšia sa len drobnosťou v názve, majú takmer rovnaké logo a namiesto pomoci pýtajú predplatné. Ukážeme si tri jednoduché kontroly, podľa ktorých spoznáte tú pravú.</t>
         </is>
       </c>
       <c r="F90" s="10" t="inlineStr"/>
@@ -3340,9 +3340,9 @@
           <t>Prezrite si kartu pravej aplikácie a tri kontroly pod ňou. Ak si chcete ChatGPT otvoriť hneď, použite tlačidlo pri svojom zariadení — otvorí sa v novom okne a o kurz neprídete.</t>
         </is>
       </c>
-      <c r="E91" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E91" s="7" t="inlineStr">
+        <is>
+          <t>Prezrite si kartu pravej aplikácie a tri kontroly pod ňou. Ak si chcete ChatGPT otvoriť hneď, kliknite na tlačidlo pri zariadení, ktoré používate. Otvorí sa v novom okne, takže o rozrobený kurz neprídete — vrátite sa doň zatvorením toho okna.</t>
         </is>
       </c>
       <c r="F91" s="10" t="inlineStr"/>
@@ -3543,9 +3543,9 @@
           <t>Takto vyzerá logo pravej aplikácie. Toto je jediné oficiálne ChatGPT.</t>
         </is>
       </c>
-      <c r="E98" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E98" s="7" t="inlineStr">
+        <is>
+          <t>Takto vyzerá logo pravej aplikácie — jednoduchý čierny alebo biely kvietok. Toto je jediné oficiálne ChatGPT; všetko ostatné s pestrofarebnými robotmi a mozgami sú napodobeniny.</t>
         </is>
       </c>
       <c r="F98" s="10" t="inlineStr"/>
@@ -3978,9 +3978,9 @@
           <t>Je to napísané priamo pod názvom aplikácie. Toto je najspoľahlivejší znak — spoľahlivejší než logo, ktoré sa dá napodobniť.</t>
         </is>
       </c>
-      <c r="E113" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>Meno vydavateľa je napísané priamo pod názvom aplikácie a musí tam byť OpenAI. Toto je najspoľahlivejší znak zo všetkých — logo sa dá napodobniť takmer dokonale, meno vydavateľa nie.</t>
         </is>
       </c>
       <c r="F113" s="10" t="inlineStr"/>
@@ -4007,9 +4007,9 @@
           <t>Ak niečo pýta peniaze už za samotné stiahnutie, je to podvod. Pravé ChatGPT sa inštaluje bezplatne.</t>
         </is>
       </c>
-      <c r="E114" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>Pravé ChatGPT sa sťahuje aj používa zadarmo. Ak od vás nejaká aplikácia pýta peniaze už za samotné stiahnutie, je to napodobenina — a vaše peniaze aj údaje o karte skončia u podvodníka.</t>
         </is>
       </c>
       <c r="F114" s="10" t="inlineStr"/>
@@ -4036,9 +4036,9 @@
           <t>Nikdy nie z odkazu v SMS, e-maile ani z reklamy. Aj keby odkaz vyzeral akokoľvek dôveryhodne.</t>
         </is>
       </c>
-      <c r="E115" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E115" s="7" t="inlineStr">
+        <is>
+          <t>Aplikácie sťahujte jedine z Google Play alebo App Store, nikdy z odkazu v SMS, e-maile či z reklamy na sociálnej sieti. A to aj vtedy, keď odkaz vyzerá úplne dôveryhodne — práve tak to podvodníci myslia.</t>
         </is>
       </c>
       <c r="F115" s="10" t="inlineStr"/>
@@ -4152,9 +4152,9 @@
           <t>Na všetko, čo robíme v tomto kurze, úplne stačí. Môžete sa pýtať, dať si vysvetliť správu aj posúdiť podozrivý e-mail. Nič platiť nemusíte.</t>
         </is>
       </c>
-      <c r="E119" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E119" s="7" t="inlineStr">
+        <is>
+          <t>Na všetko, čo v tomto kurze robíme, úplne stačí. Môžete sa pýtať, dať si vysvetliť list z úradu aj posúdiť podozrivý e-mail. Nemusíte zadávať kartu ani nič platiť — a nikdy sa vám z nej sama nestane platená.</t>
         </is>
       </c>
       <c r="F119" s="10" t="inlineStr"/>
@@ -4181,9 +4181,9 @@
           <t>Stojí okolo 20 € mesačne a dáva rýchlejšie odpovede a novšie funkcie. Pre naše účely nie je potrebná.</t>
         </is>
       </c>
-      <c r="E120" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E120" s="7" t="inlineStr">
+        <is>
+          <t>Stojí okolo 20 € mesačne a ponúka rýchlejšie odpovede a novinky navyše. Pre to, čo potrebujeme my, nie je potrebná — pokojne ju nechajte tak.</t>
         </is>
       </c>
       <c r="F120" s="10" t="inlineStr"/>
@@ -4210,9 +4210,9 @@
           <t>Predplatné sa platí jedine priamo v aplikácii alebo na chatgpt.com. Ak vám niekto ponúka „predplatné ChatGPT“ e-mailom, cez SMS alebo v reklame na sociálnej sieti, je to podvod — presne ten typ, aký sme si ukazovali.</t>
         </is>
       </c>
-      <c r="E121" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>Ak by ste sa niekedy rozhodli platenú verziu predsa len vyskúšať, platí sa jedine priamo v aplikácii alebo na stránke chatgpt.com. Ponuka „predplatného ChatGPT“, ktorá vám príde e-mailom, cez SMS alebo v reklame na sociálnej sieti, je vždy podvod — presne ten typ, aký si v kurze ukazujeme.</t>
         </is>
       </c>
       <c r="F121" s="10" t="inlineStr"/>
@@ -4239,9 +4239,9 @@
           <t>Pri registrácii vás ChatGPT požiada o e-mailovú adresu — to je v poriadku a bezpečné. Heslo si však vymyslite nové, nikdy nepoužívajte to isté, aké máte do banky alebo do e-mailu.</t>
         </is>
       </c>
-      <c r="E122" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E122" s="7" t="inlineStr">
+        <is>
+          <t>Pri prvom prihlásení vás ChatGPT požiada o e-mailovú adresu. To je bežné a bezpečné — potrebuje vedieť, komu patria vaše rozhovory. Heslo si však vymyslite úplne nové. Nikdy nepoužívajte to isté, aké máte do banky alebo do e-mailu; keby sa jedno prezradilo, podvodník by mal rovno aj to druhé.</t>
         </is>
       </c>
       <c r="F122" s="10" t="inlineStr"/>
@@ -4297,9 +4297,9 @@
           <t>Obrazovku už poznáte. Teraz si prejdime, čo na nej urobíte — píše sa s ňou rovnako ako SMS správa.</t>
         </is>
       </c>
-      <c r="E124" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E124" s="11" t="inlineStr">
+        <is>
+          <t>Obrazovku už poznáte. Teraz si prejdeme, čo na nej postupne urobíte. Nie je to nič zložité — píše sa s ňou rovnako ako SMS správa vnúčaťu.</t>
         </is>
       </c>
       <c r="F124" s="10" t="inlineStr"/>
@@ -4326,9 +4326,9 @@
           <t>Päť krokov je zámerne pomiešaných. Klikajte na ne &lt;strong&gt;v poradí, v akom by ste ich naozaj robili&lt;/strong&gt; — začnite tým, čo urobíte úplne ako prvé.</t>
         </is>
       </c>
-      <c r="E125" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E125" s="11" t="inlineStr">
+        <is>
+          <t>Päť krokov je zámerne pomiešaných. Klikajte na ne &lt;strong&gt;v poradí, v akom by ste ich naozaj robili&lt;/strong&gt; — začnite tým, čo urobíte úplne ako prvé. Ak sa pomýlite, jednoducho skúsite znova.</t>
         </is>
       </c>
       <c r="F125" s="10" t="inlineStr"/>
@@ -4384,9 +4384,9 @@
           <t>Dole na obrazovke nájdete okienko na písanie — rovnaké ako pri SMS.</t>
         </is>
       </c>
-      <c r="E127" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E127" s="11" t="inlineStr">
+        <is>
+          <t>Dole na obrazovke nájdite okienko na písanie — vyzerá rovnako ako pri písaní SMS.</t>
         </is>
       </c>
       <c r="F127" s="10" t="inlineStr"/>
@@ -4413,9 +4413,9 @@
           <t>Napíšte otázku celou vetou, ako by ste ju položili človeku.</t>
         </is>
       </c>
-      <c r="E128" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E128" s="11" t="inlineStr">
+        <is>
+          <t>Napíšte otázku celou vetou, tak ako by ste ju položili človeku.</t>
         </is>
       </c>
       <c r="F128" s="10" t="inlineStr"/>
@@ -4442,9 +4442,9 @@
           <t>Stlačte šípku (odoslať) a počkajte pár sekúnd na odpoveď.</t>
         </is>
       </c>
-      <c r="E129" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E129" s="11" t="inlineStr">
+        <is>
+          <t>Stlačte šípku na odoslanie a počkajte pár sekúnd, kým sa odpoveď vypíše.</t>
         </is>
       </c>
       <c r="F129" s="10" t="inlineStr"/>
@@ -4500,9 +4500,9 @@
           <t>Presne takto to bude vyzerať aj u vás doma. Celé to trvá menej než minútu.</t>
         </is>
       </c>
-      <c r="E131" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E131" s="11" t="inlineStr">
+        <is>
+          <t>Presne takto to bude vyzerať aj u vás doma. Celé to trvá menej než minútu a nič viac na začiatok vedieť nemusíte.</t>
         </is>
       </c>
       <c r="F131" s="10" t="inlineStr"/>
@@ -4529,9 +4529,9 @@
           <t>V ChatGPT sa nedá nič pokaziť. Žiadne tlačidlo nič nezmaže vo vašom mobile ani účte.</t>
         </is>
       </c>
-      <c r="E132" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E132" s="11" t="inlineStr">
+        <is>
+          <t>V ChatGPT sa nedá nič pokaziť. Žiadne tlačidlo vám nič nezmaže v telefóne, v e-maile ani v banke — v najhoršom prípade dostanete odpoveď, ktorá vás nezaujíma, a spýtate sa inak.</t>
         </is>
       </c>
       <c r="F132" s="10" t="inlineStr"/>
@@ -4587,9 +4587,9 @@
           <t>Otázke pre umelú inteligenciu sa hovorí „prompt“. Platí jednoduché pravidlo: čím presnejšia otázka, tým užitočnejšia odpoveď.</t>
         </is>
       </c>
-      <c r="E134" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E134" s="7" t="inlineStr">
+        <is>
+          <t>Otázke, ktorú položíte umelej inteligencii, sa hovorí „prompt“. Platí pri nej jednoduché pravidlo: čím presnejšie sa opýtate, tým užitočnejšiu odpoveď dostanete.</t>
         </is>
       </c>
       <c r="F134" s="10" t="inlineStr"/>
@@ -4616,9 +4616,9 @@
           <t>Uvidíte &lt;strong&gt;tri dvojice otázok&lt;/strong&gt;. Pri každej kliknite na tú, ktorá je podľa vás pre AI lepšia. Hneď vám vysvetlíme, prečo.</t>
         </is>
       </c>
-      <c r="E135" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E135" s="7" t="inlineStr">
+        <is>
+          <t>Uvidíte &lt;strong&gt;tri dvojice otázok&lt;/strong&gt;. Pri každej kliknite na tú, ktorá je podľa vás pre umelú inteligenciu lepšia. Hneď vám vysvetlíme, prečo — a čím sa tá druhá pokazila.</t>
         </is>
       </c>
       <c r="F135" s="10" t="inlineStr"/>
@@ -4645,9 +4645,9 @@
           <t>Je to ako u lekára: „bolí ma tu, od včera, po jedle“ je lepšie než len „je mi zle“.</t>
         </is>
       </c>
-      <c r="E136" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E136" s="7" t="inlineStr">
+        <is>
+          <t>Je to ako u lekára. Keď poviete „je mi zle“, dostanete všeobecnú radu. Keď poviete „bolí ma tu, od včera, vždy po jedle“, dostanete odpoveď, ktorá vám naozaj pomôže. S umelou inteligenciou je to úplne rovnaké.</t>
         </is>
       </c>
       <c r="F136" s="10" t="inlineStr"/>
@@ -4848,9 +4848,9 @@
           <t>AI nevie, kto ste ani čo sa stalo. Konkrétny popis dá konkrétnu odpoveď.</t>
         </is>
       </c>
-      <c r="E143" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E143" s="7" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia nevie, kto ste, ani čo sa vám stalo — vidí len to, čo napíšete. Keď opíšete situáciu konkrétne, dostanete konkrétnu odpoveď namiesto všeobecných rád.</t>
         </is>
       </c>
       <c r="F143" s="10" t="inlineStr"/>
@@ -4877,9 +4877,9 @@
           <t>Jedno slovo nestačí — opíšte situáciu tak, ako by ste ju vysvetlili susedovi.</t>
         </is>
       </c>
-      <c r="E144" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E144" s="7" t="inlineStr">
+        <is>
+          <t>Jedno slovo alebo krátka otázka nestačí. Opíšte situáciu tak, ako by ste ju vysvetlili susedovi cez plot — kto vám čo ponúka, za koľko a čo vám na tom nesedí.</t>
         </is>
       </c>
       <c r="F144" s="10" t="inlineStr"/>
@@ -4906,9 +4906,9 @@
           <t>AI vám nerozhodne za vás, ale pomôže spýtať sa na správne veci.</t>
         </is>
       </c>
-      <c r="E145" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E145" s="7" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia za vás nerozhodne a ani by nemala. Zato vám pripraví otázky, ktoré sa oplatí položiť — a práve pri nich sa podvodník zvyčajne prezradí.</t>
         </is>
       </c>
       <c r="F145" s="10" t="inlineStr"/>
@@ -4935,9 +4935,9 @@
           <t>Užitočná rada: na koniec otázky pridajte „Vysvetli mi to jednoducho, ako seniorovi.“</t>
         </is>
       </c>
-      <c r="E146" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E146" s="7" t="inlineStr">
+        <is>
+          <t>Užitočná rada na záver: na koniec otázky pokojne pridajte vetu „Vysvetli mi to jednoducho, bez odborných slov.“ Odpoveď potom bude kratšia a zrozumiteľnejšia. Túto vetu môžete použiť pri každej otázke.</t>
         </is>
       </c>
       <c r="F146" s="10" t="inlineStr"/>
@@ -5254,9 +5254,9 @@
           <t>Overovanie nie je prejav nedôvery — je to obyčajný zdravý rozum, rovnaký, aký by ste použili pri rade od susedy.</t>
         </is>
       </c>
-      <c r="E157" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E157" s="7" t="inlineStr">
+        <is>
+          <t>Overovanie nie je prejav nedôvery, je to obyčajný zdravý rozum. Keď vám susedka poradí, kde kúpiť lacnejšie lieky, tiež sa najskôr pozriete sami. S umelou inteligenciou je to presne rovnaké.</t>
         </is>
       </c>
       <c r="F157" s="10" t="inlineStr"/>
@@ -5283,9 +5283,9 @@
           <t>Kliknite postupne na &lt;strong&gt;všetky tri kľúče&lt;/strong&gt;. Za každým sa skrýva jedno pravidlo, ako si odpoveď AI overiť.</t>
         </is>
       </c>
-      <c r="E158" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E158" s="7" t="inlineStr">
+        <is>
+          <t>Kliknite postupne na &lt;strong&gt;všetky tri kľúče&lt;/strong&gt;. Za každým sa skrýva jedno pravidlo, ako si odpoveď od umelej inteligencie overiť. Sú krátke a zapamätáte si ich hneď.</t>
         </is>
       </c>
       <c r="F158" s="10" t="inlineStr"/>
@@ -5399,9 +5399,9 @@
           <t>Čísla, dátumy či telefónne čísla skontrolujte na oficiálnej stránke banky alebo úradu.</t>
         </is>
       </c>
-      <c r="E162" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E162" s="7" t="inlineStr">
+        <is>
+          <t>Konkrétne údaje — čísla, dátumy, telefónne linky — si prezrite ešte na oficiálnej stránke banky alebo úradu. Práve tieto si umelá inteligencia najčastejšie vymyslí, a znie pritom úplne isto.</t>
         </is>
       </c>
       <c r="F162" s="10" t="inlineStr"/>
@@ -5428,9 +5428,9 @@
           <t>„Odkiaľ to vieš? Kde si to môžem overiť?“ Ak AI zdroj neuvedie, buďte opatrní.</t>
         </is>
       </c>
-      <c r="E163" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E163" s="7" t="inlineStr">
+        <is>
+          <t>Pokojne sa jej priamo opýtajte: „Odkiaľ to vieš? Kde si to môžem overiť?“ Ak zdroj neuvedie alebo začne odpovedať vyhýbavo, berte odpoveď len ako názor, nie ako fakt.</t>
         </is>
       </c>
       <c r="F163" s="10" t="inlineStr"/>
@@ -5457,9 +5457,9 @@
           <t>Nikdy nerobte finančné rozhodnutie len na základe odpovede AI. AI radí, človek rozhoduje.</t>
         </is>
       </c>
-      <c r="E164" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E164" s="7" t="inlineStr">
+        <is>
+          <t>Nikdy sa nerozhodujte o peniazoch len na základe toho, čo napísala umelá inteligencia. Nech znie akokoľvek presvedčivo, pri väčšej sume sa opýtajte aj svojho bankára alebo niekoho blízkeho. AI radí, človek rozhoduje.</t>
         </is>
       </c>
       <c r="F164" s="10" t="inlineStr"/>
@@ -5486,9 +5486,9 @@
           <t>Novšie verzie AI halucinujú menej často než staršie, no úplne sa toho zbaviť zatiaľ nepodarilo.</t>
         </is>
       </c>
-      <c r="E165" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E165" s="7" t="inlineStr">
+        <is>
+          <t>Novšie verzie umelej inteligencie si vymýšľajú menej často než tie staršie, ale úplne sa toho zbaviť zatiaľ nepodarilo. Preto pravidlo „dôležité si overím“ platí aj naďalej — a bude platiť ešte dlho.</t>
         </is>
       </c>
       <c r="F165" s="10" t="inlineStr"/>
@@ -5544,9 +5544,9 @@
           <t>Zopakujme si, čo sme sa doteraz naučili o umelej inteligencii.</t>
         </is>
       </c>
-      <c r="E167" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E167" s="11" t="inlineStr">
+        <is>
+          <t>Zopakujme si krátko, čo už o umelej inteligencii vieme. Nie je to skúška — ide len o to, aby vám tie tri veci utkveli.</t>
         </is>
       </c>
       <c r="F167" s="10" t="inlineStr"/>
@@ -5573,9 +5573,9 @@
           <t>Tri rýchle otázky. Pri každej kliknite &lt;strong&gt;Áno&lt;/strong&gt; alebo &lt;strong&gt;Nie&lt;/strong&gt; — hneď sa dozviete, či ste odpovedali správne, aj prečo.</t>
         </is>
       </c>
-      <c r="E168" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E168" s="11" t="inlineStr">
+        <is>
+          <t>Tri rýchle otázky. Pri každej kliknite &lt;strong&gt;Áno&lt;/strong&gt; alebo &lt;strong&gt;Nie&lt;/strong&gt; — hneď sa dozviete, či ste sa trafili, aj prečo je odpoveď taká. Nesprávna odpoveď nič nepokazí.</t>
         </is>
       </c>
       <c r="F168" s="10" t="inlineStr"/>
@@ -5602,9 +5602,9 @@
           <t>AI je pomocník: vysvetľuje, zhŕňa a upozorňuje na riziká.</t>
         </is>
       </c>
-      <c r="E169" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E169" s="11" t="inlineStr">
+        <is>
+          <t>Umelá inteligencia je pomocník: vysvetlí, zhrnie a upozorní na riziká.</t>
         </is>
       </c>
       <c r="F169" s="10" t="inlineStr"/>
@@ -5660,9 +5660,9 @@
           <t>Pri dôležitých faktoch platí — najprv overiť, potom konať.</t>
         </is>
       </c>
-      <c r="E171" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E171" s="11" t="inlineStr">
+        <is>
+          <t>Pri dôležitých údajoch platí jednoduché poradie — najprv overiť, potom konať.</t>
         </is>
       </c>
       <c r="F171" s="10" t="inlineStr"/>
@@ -5863,9 +5863,9 @@
           <t>Nie. AI nemá prístup k žiadnym vašim účtom ani súkromným údajom, pokiaľ jej ich sami nenapíšete. A práve preto jej ich nikdy nepíšeme.</t>
         </is>
       </c>
-      <c r="E178" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E178" s="11" t="inlineStr">
+        <is>
+          <t>Nie. Umelá inteligencia sa do vášho bankového účtu nevidí a nevie s ním nič urobiť — nemá k nemu žiadny prístup. Vedieť o vás môže len to, čo jej sami napíšete. A práve preto jej svoje čísla účtov, heslá a kódy nikdy nepíšeme.</t>
         </is>
       </c>
       <c r="F178" s="10" t="inlineStr"/>
@@ -5892,9 +5892,9 @@
           <t>Nie. V ChatGPT sa nedá nič nenávratne zmazať ani pokaziť — pokojne skúšajte, čo vás zaujíma. Nič vo vašom mobile ani účte to nezmení.</t>
         </is>
       </c>
-      <c r="E179" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E179" s="11" t="inlineStr">
+        <is>
+          <t>Nie. V ChatGPT sa nedá nič nenávratne zmazať ani pokaziť. Pokojne skúšajte, pýtajte sa aj hlúposti a mažte rozhovory — vo vašom telefóne, e-maile ani v banke sa tým nič nezmení. Preto sa nemusíte báť čokoľvek vyskúšať.</t>
         </is>
       </c>
       <c r="F179" s="10" t="inlineStr"/>
@@ -5921,9 +5921,9 @@
           <t>Áno. AI sa občas mýli a tvári sa pritom presvedčivo — preto dôležité informácie vždy overte aj z druhého zdroja.</t>
         </is>
       </c>
-      <c r="E180" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E180" s="11" t="inlineStr">
+        <is>
+          <t>Áno, a to je najdôležitejšia vec z celej tejto časti. Umelá inteligencia sa občas mýli a tvári sa pritom rovnako isto ako inokedy. Preto si dôležité informácie vždy overte aj z druhého zdroja.</t>
         </is>
       </c>
       <c r="F180" s="10" t="inlineStr"/>
@@ -5979,9 +5979,9 @@
           <t>Skôr než sa pustíme do skutočných podvodov, pomenujme si ich. Všetky tri majú spoločné jedno — chcú od vás vylákať údaje alebo peniaze.</t>
         </is>
       </c>
-      <c r="E182" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E182" s="7" t="inlineStr">
+        <is>
+          <t>Skôr než sa pustíme do skutočných podvodov, pomenujme si ich. Budete tie slová počuť v správach aj od banky, tak nech viete, o čom je reč. Všetky tri majú spoločné jedno: chcú z vás dostať údaje alebo peniaze.</t>
         </is>
       </c>
       <c r="F182" s="10" t="inlineStr"/>
@@ -6008,9 +6008,9 @@
           <t>Kliknite na &lt;strong&gt;pojem vľavo&lt;/strong&gt; a potom na &lt;strong&gt;vysvetlenie vpravo&lt;/strong&gt;, ktoré k nemu patrí.</t>
         </is>
       </c>
-      <c r="E183" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E183" s="7" t="inlineStr">
+        <is>
+          <t>Kliknite na &lt;strong&gt;pojem vľavo&lt;/strong&gt; a potom na &lt;strong&gt;vysvetlenie vpravo&lt;/strong&gt;, ktoré k nemu podľa vás patrí. Ak sa trafíte, spojí ich čiara.</t>
         </is>
       </c>
       <c r="F183" s="10" t="inlineStr"/>
@@ -6124,9 +6124,9 @@
           <t>Podvodný e-mail, ktorý sa tvári ako správa od banky a chce vylákať vaše údaje.</t>
         </is>
       </c>
-      <c r="E187" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E187" s="7" t="inlineStr">
+        <is>
+          <t>Podvodný e-mail, ktorý sa tvári ako správa od banky a chce z vás dostať prihlasovacie údaje.</t>
         </is>
       </c>
       <c r="F187" s="10" t="inlineStr"/>
@@ -6211,9 +6211,9 @@
           <t>Phishing chodí e-mailom. Slovo vzniklo z anglického „fishing“ — rybolov, lebo podvodníci „lovia“ vaše údaje.</t>
         </is>
       </c>
-      <c r="E190" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>Phishing chodí e-mailom. Slovo vzniklo z anglického „fishing“, teda rybolov — podvodníci hodia návnadu tisíckam ľudí naraz a čakajú, kto sa chytí. Stačí im pritom jediný z tisíca.</t>
         </is>
       </c>
       <c r="F190" s="10" t="inlineStr"/>
@@ -6240,9 +6240,9 @@
           <t>Vishing prebieha po telefóne. Písmeno „v“ je z anglického „voice“ — hlas.</t>
         </is>
       </c>
-      <c r="E191" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E191" s="7" t="inlineStr">
+        <is>
+          <t>Vishing prebieha po telefóne. Písmeno „v“ je z anglického „voice“, teda hlas. Je nebezpečnejší než e-mail, lebo živý človek na vás dokáže tlačiť a nedá vám čas rozmyslieť si to.</t>
         </is>
       </c>
       <c r="F191" s="10" t="inlineStr"/>
@@ -6269,9 +6269,9 @@
           <t>Smishing chodí ako SMS. Najčastejšie ide o „nedoručený balík“ s malým poplatkom.</t>
         </is>
       </c>
-      <c r="E192" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>Smishing chodí ako SMS správa. Najčastejšie ide o „nedoručený balík“, ktorý stačí doplatiť pár centov — a práve pri tom zaplatení odovzdáte údaje o svojej karte.</t>
         </is>
       </c>
       <c r="F192" s="10" t="inlineStr"/>
@@ -6298,9 +6298,9 @@
           <t>Bez ohľadu na to, ktorý z nich vás zastihne, obrana je vždy rovnaká: spomaliť, neklikať a overiť si to.</t>
         </is>
       </c>
-      <c r="E193" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E193" s="7" t="inlineStr">
+        <is>
+          <t>Nemusíte si tie slová pamätať naspamäť. Dôležité je, že obrana je pri všetkých troch rovnaká: spomaliť, na nič neklikať a overiť si to na čísle alebo stránke, ktorú si nájdete sami.</t>
         </is>
       </c>
       <c r="F193" s="10" t="inlineStr"/>
@@ -7139,9 +7139,9 @@
           <t>Tento e-mail naozaj chodil klientom slovenskej banky. Vyskúšajme si na ňom, čo sme sa práve naučili.</t>
         </is>
       </c>
-      <c r="E222" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E222" s="11" t="inlineStr">
+        <is>
+          <t>Tento e-mail naozaj chodil klientom slovenskej banky — nie je vymyslený pre kurz. Vyskúšajme si na ňom, čo sme sa pred chvíľou naučili. Tentoraz už bez nápovedy, ktorý znak je ktorý.</t>
         </is>
       </c>
       <c r="F222" s="10" t="inlineStr"/>
@@ -7168,9 +7168,9 @@
           <t>Nájdite &lt;strong&gt;4 varovné znaky&lt;/strong&gt; — kliknite postupne na podčiarknuté časti textu. Všimnite si aj adresu odosielateľa hore, tá je tiež nezvyčajná.</t>
         </is>
       </c>
-      <c r="E223" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E223" s="11" t="inlineStr">
+        <is>
+          <t>Nájdite &lt;strong&gt;4 varovné znaky&lt;/strong&gt; — kliknite postupne na podčiarknuté časti textu. Pozrite sa aj na adresu odosielateľa úplne hore; aj tá o e-maile veľa prezradí.</t>
         </is>
       </c>
       <c r="F223" s="10" t="inlineStr"/>
@@ -7284,9 +7284,9 @@
           <t>Všeobecné oslovenie „Vážený zákazník“ — skutočná banka pozná vaše meno a oslovila by vás ním.</t>
         </is>
       </c>
-      <c r="E227" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E227" s="11" t="inlineStr">
+        <is>
+          <t>Oslovenie „Vážený zákazník“ znamená, že odosielateľ vaše meno nepozná. Skutočná banka vás v e-maile osloví menom, prípadne uvedie posledné štyri číslice vášho účtu — vie predsa, komu píše.</t>
         </is>
       </c>
       <c r="F227" s="10" t="inlineStr"/>
@@ -7313,9 +7313,9 @@
           <t>Strach a časový tlak — tvrdenie, že účet je „dočasne zablokovaný“.</t>
         </is>
       </c>
-      <c r="E228" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E228" s="11" t="inlineStr">
+        <is>
+          <t>Tvrdenie, že účet je „dočasne zablokovaný“, má vo vás vyvolať strach. Vystrašený človek prestane rozmýšľať a chce problém rýchlo vyriešiť — presne s tým podvodník počíta. Ak by banka váš účet naozaj zablokovala, dozviete sa to v aplikácii alebo vám zavolá.</t>
         </is>
       </c>
       <c r="F228" s="10" t="inlineStr"/>
@@ -7342,9 +7342,9 @@
           <t>Naliehavá výzva „okamžite dokončite overenie“ — má vás donútiť konať bez rozmýšľania.</t>
         </is>
       </c>
-      <c r="E229" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E229" s="11" t="inlineStr">
+        <is>
+          <t>Výzva „okamžite dokončite overenie“ vás má prinútiť konať bez rozmýšľania. Všimnite si, že vám nedáva žiadnu inú možnosť — žiadne „zavolajte nám“, žiadne „navštívte pobočku“. Len to jedno tlačidlo.</t>
         </is>
       </c>
       <c r="F229" s="10" t="inlineStr"/>
@@ -7371,9 +7371,9 @@
           <t>Automaticky generovaný e-mail bez podpisu konkrétnej osoby — typické pre hromadné podvodné rozposielanie.</t>
         </is>
       </c>
-      <c r="E230" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E230" s="11" t="inlineStr">
+        <is>
+          <t>Veta o automaticky vygenerovanom e-maile bez podpisu konkrétneho človeka či oddelenia je typická pre hromadné rozposielanie. Podvodník neposiela správu vám, ale desiatkam tisíc ľudí naraz.</t>
         </is>
       </c>
       <c r="F230" s="10" t="inlineStr"/>
@@ -7400,9 +7400,9 @@
           <t>Adresa odosielateľa (no-reply-2247@livemail.co.uk) je dlhý nezmyselný reťazec a nekončí na doméne skutočnej banky. Presne takýto e-mail môžete odfotiť a poslať do AI s otázkou: „Je to podvod?“</t>
         </is>
       </c>
-      <c r="E231" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E231" s="11" t="inlineStr">
+        <is>
+          <t>Pozrite sa na adresu odosielateľa: no-reply-2247@livemail.co.uk. Je to nezmyselný reťazec a nekončí názvom banky — skutočná banka píše z adresy, v ktorej je jej meno. Ak si nie ste istý, e-mail odfoťte alebo prepíšte do ChatGPT a opýtajte sa: „Je toto podvod?“ A potom zavolajte do banky na číslo zo svojej karty.</t>
         </is>
       </c>
       <c r="F231" s="10" t="inlineStr"/>
@@ -7429,9 +7429,9 @@
           <t>Skutočný podvodný e-mail, ktorý chodil klientom VÚB banky. Odosielateľ nie je banka, len sa za ňu vydáva.</t>
         </is>
       </c>
-      <c r="E232" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E232" s="11" t="inlineStr">
+        <is>
+          <t>Toto je skutočný podvodný e-mail, ktorý chodil klientom VÚB banky. Vyzerá dôveryhodne vrátane loga — ale odosielateľ nie je banka, len sa za ňu vydáva.</t>
         </is>
       </c>
       <c r="F232" s="10" t="inlineStr"/>
@@ -7487,9 +7487,9 @@
           <t>Pozor — nie každý podvod straší. Tento naopak sľubuje peniaze, a práve tým je nebezpečný.</t>
         </is>
       </c>
-      <c r="E234" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E234" s="7" t="inlineStr">
+        <is>
+          <t>Pozor, nie každý podvod straší. Tento naopak sľubuje peniaze — a práve tým je nebezpečný. Pri dobrej správe totiž človek stráca ostražitosť oveľa ľahšie než pri hrozbe.</t>
         </is>
       </c>
       <c r="F234" s="10" t="inlineStr"/>
@@ -7516,9 +7516,9 @@
           <t>Nájdite &lt;strong&gt;3 varovné znaky&lt;/strong&gt;. Kliknite na podčiarknuté časti a všímajte si, ako podvodník mieša sľub peňazí so žiadosťou o údaje.</t>
         </is>
       </c>
-      <c r="E235" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E235" s="7" t="inlineStr">
+        <is>
+          <t>Nájdite &lt;strong&gt;3 varovné znaky&lt;/strong&gt;. Kliknite na podčiarknuté časti a všímajte si, ako podvodník sľub peňazí šikovne mieša so žiadosťou o údaje z karty.</t>
         </is>
       </c>
       <c r="F235" s="10" t="inlineStr"/>
@@ -7632,9 +7632,9 @@
           <t>Nečakaná „vratka“ 490 € — sľub peňazí je návnada, nikto vám len tak neposiela stovky eur.</t>
         </is>
       </c>
-      <c r="E239" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E239" s="7" t="inlineStr">
+        <is>
+          <t>Nečakaný preplatok 490 € je návnada. Nikto vám len tak neposiela stovky eur — a keby ste naozaj mali na niečo nárok, dozvedeli by ste sa to listom alebo v poisťovni, nie prekvapivým e-mailom.</t>
         </is>
       </c>
       <c r="F239" s="10" t="inlineStr"/>
@@ -7661,9 +7661,9 @@
           <t>Text je preložený strojovo — všimnite si francúzske „carte bancaire“, ktoré tam vôbec nepatrí.</t>
         </is>
       </c>
-      <c r="E240" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E240" s="7" t="inlineStr">
+        <is>
+          <t>Text je preložený strojom — všimnite si francúzske „carte bancaire“, ktoré do slovenskej vety vôbec nepatrí. Znamená to, že rovnaká správa sa rozposiela po celej Európe a niekto ju len narýchlo preložil.</t>
         </is>
       </c>
       <c r="F240" s="10" t="inlineStr"/>
@@ -7690,9 +7690,9 @@
           <t>Žiada údaje o karte — poisťovňa vracia peniaze na účet, nikdy si nepýta kartu cez e-mail.</t>
         </is>
       </c>
-      <c r="E241" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E241" s="7" t="inlineStr">
+        <is>
+          <t>Správa pýta číslo platobnej karty. Toto je tá najdôležitejšia vec: peniaze sa vracajú na účet, na ktorý ste platili, a na to nikto nepotrebuje vašu kartu. Kto od vás pýta jej číslo, nechce vám peniaze poslať — chce ich z nej vybrať.</t>
         </is>
       </c>
       <c r="F241" s="10" t="inlineStr"/>
@@ -7719,9 +7719,9 @@
           <t>Ako si to overiť: zavolajte priamo poisťovni na oficiálne číslo z jej webovej stránky — nikdy nie na číslo uvedené v podozrivom e-maile.</t>
         </is>
       </c>
-      <c r="E242" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E242" s="7" t="inlineStr">
+        <is>
+          <t>Ako si to overiť: zavolajte priamo poisťovni na číslo, ktoré nájdete na jej oficiálnej stránke alebo na svojom preukaze poistenca. Nikdy nevolajte na číslo uvedené v podozrivom e-maile — tam vám zdvihne ten istý podvodník.</t>
         </is>
       </c>
       <c r="F242" s="10" t="inlineStr"/>
@@ -7748,9 +7748,9 @@
           <t>Skutočná falošná „faktúra o náhrade“ vydávajúca sa za zdravotnú poisťovňu. Žiadna poisťovňa takto peniaze nevracia.</t>
         </is>
       </c>
-      <c r="E243" s="9" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E243" s="7" t="inlineStr">
+        <is>
+          <t>Skutočná falošná „faktúra o náhrade“, ktorá sa vydáva za zdravotnú poisťovňu. Žiadna poisťovňa peniaze takto nevracia a údaje o karte cez e-mail nikdy nežiada.</t>
         </is>
       </c>
       <c r="F243" s="10" t="inlineStr"/>
@@ -7806,9 +7806,9 @@
           <t>Najrozšírenejší podvod na Slovensku. Funguje preto, že takmer každý dnes niečo očakáva poštou.</t>
         </is>
       </c>
-      <c r="E245" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E245" s="11" t="inlineStr">
+        <is>
+          <t>Toto je dnes najrozšírenejší podvod na Slovensku. Funguje preto, že takmer každý niečo čaká poštou — a keď človek naozaj čaká balík, správu si ani poriadne neprečíta.</t>
         </is>
       </c>
       <c r="F245" s="10" t="inlineStr"/>
@@ -7835,9 +7835,9 @@
           <t>Nájdite &lt;strong&gt;4 varovné znaky&lt;/strong&gt;. Kliknite na podčiarknuté časti — všimnite si najmä, aká drobná je požadovaná suma.</t>
         </is>
       </c>
-      <c r="E246" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E246" s="11" t="inlineStr">
+        <is>
+          <t>Nájdite &lt;strong&gt;4 varovné znaky&lt;/strong&gt;. Kliknite na podčiarknuté časti a všimnite si najmä, aká drobná je požadovaná suma — to nie je náhoda.</t>
         </is>
       </c>
       <c r="F246" s="10" t="inlineStr"/>
@@ -7951,9 +7951,9 @@
           <t>Malý poplatok 3,59 € — drobná suma nevzbudí podozrenie. Podvodníkom však nejde o tie tri eurá, ale o údaje z vašej karty.</t>
         </is>
       </c>
-      <c r="E250" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E250" s="11" t="inlineStr">
+        <is>
+          <t>Poplatok 3,59 € je zámerne drobný — pri takej sume človek nezaváha a zaplatí. Podvodníkom pritom o tie tri eurá vôbec nejde. Ide im o číslo vašej karty, ktoré pri platbe zadáte; z neho potom zmizne oveľa viac.</t>
         </is>
       </c>
       <c r="F250" s="10" t="inlineStr"/>
@@ -7980,9 +7980,9 @@
           <t>Chyby v slovenčine — „aby ste zaplatili po prijatí tento správy“ a chýbajúce mäkčene v úvode.</t>
         </is>
       </c>
-      <c r="E251" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E251" s="11" t="inlineStr">
+        <is>
+          <t>Chyby v slovenčine — „aby ste zaplatili po prijatí tento správy“ a chýbajúce mäkčene hneď v úvode. Slovenská pošta píše po slovensky správne. Pozor však: dnes už podvodníci používajú prekladače aj umelú inteligenciu, takže bezchybný text ešte nič nezaručuje.</t>
         </is>
       </c>
       <c r="F251" s="10" t="inlineStr"/>
@@ -8009,9 +8009,9 @@
           <t>Tlačidlo „Kliknite tu“ vedie na falošnú platobnú stránku, ktorá vyzerá ako tá skutočná.</t>
         </is>
       </c>
-      <c r="E252" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E252" s="11" t="inlineStr">
+        <is>
+          <t>Tlačidlo „Kliknite tu“ vedie na falošnú platobnú stránku. Býva verná kópia tej skutočnej vrátane loga, takže sa na nej nedá spoznať nič podozrivé — všetko, čo tam zadáte, ide rovno podvodníkovi.</t>
         </is>
       </c>
       <c r="F252" s="10" t="inlineStr"/>
@@ -8038,9 +8038,9 @@
           <t>Adresa odosielateľa končí na „.br“ — to je Brazília, nie slovenská pošta.</t>
         </is>
       </c>
-      <c r="E253" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E253" s="11" t="inlineStr">
+        <is>
+          <t>Adresa odosielateľa končí na „.br“, čo je skratka Brazílie. Slovenská pošta píše z adresy končiacej na .sk. Koncovka adresy je maličkosť, ktorú si takmer nikto nevšimne — a pritom prezradí podvod za dve sekundy.</t>
         </is>
       </c>
       <c r="F253" s="10" t="inlineStr"/>
@@ -8067,9 +8067,9 @@
           <t>Čakáte naozaj balík? Sledovacie číslo si zadajte priamo na oficiálnej stránke pošty alebo prepravcu — nikdy nie cez odkaz zo správy.</t>
         </is>
       </c>
-      <c r="E254" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E254" s="11" t="inlineStr">
+        <is>
+          <t>Naozaj čakáte balík? Otvorte si stránku pošty alebo prepravcu sami a zadajte tam sledovacie číslo z potvrdenia objednávky. Nikdy nie cez odkaz zo správy. A pamätajte: za doručenie balíka sa nikdy nedopláca cez odkaz v SMS ani v e-maile.</t>
         </is>
       </c>
       <c r="F254" s="10" t="inlineStr"/>
@@ -8096,9 +8096,9 @@
           <t>Skutočný podvodný e-mail vydávajúci sa za Slovenskú poštu. Adresa odosielateľa a drobný poplatok sú typickým vzorom tohto podvodu.</t>
         </is>
       </c>
-      <c r="E255" s="13" t="inlineStr">
-        <is>
-          <t>— doplním —</t>
+      <c r="E255" s="11" t="inlineStr">
+        <is>
+          <t>Skutočný podvodný e-mail, ktorý sa vydáva za Slovenskú poštu. Cudzia adresa odosielateľa a drobný poplatok sú pre tento podvod typické — keď ich raz uvidíte, spoznáte ho už vždy.</t>
         </is>
       </c>
       <c r="F255" s="10" t="inlineStr"/>

</xml_diff>